<commit_message>
Update model outputs 2026-07-11 11:55:52
</commit_message>
<xml_diff>
--- a/files/NRLW_upcoming_projections.xlsx
+++ b/files/NRLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,34 +44,52 @@
     <t xml:space="preserve">Weather Applied</t>
   </si>
   <si>
+    <t xml:space="preserve">cronulla-sutherland sharks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane broncos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain (Primary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No - primary model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted (Reference)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference only - heuristic -0.3 total pts/mm, cap +/-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">canterbury bankstown bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast titans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north queensland cowboys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wests tigers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney roosters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">newcastle knights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">canberra raiders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">warriors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st george illawarra dragons</t>
+  </si>
+  <si>
     <t xml:space="preserve">parramatta eels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wests tigers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">commbank stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain (Primary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No - primary model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather Adjusted (Reference)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference only - heuristic -0.3 total pts/mm, cap +/-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">warriors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">canterbury bankstown bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fmg stadium waikato</t>
   </si>
 </sst>
 </file>
@@ -410,9 +428,9 @@
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="4.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="15.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="29.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="19.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="29.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="5.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="28.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
@@ -454,7 +472,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46208</v>
+        <v>46212</v>
       </c>
       <c r="B2"/>
       <c r="C2" t="s">
@@ -463,28 +481,26 @@
       <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2"/>
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>19.1534851448814</v>
+      </c>
+      <c r="I2" t="n">
+        <v>39.9813771431375</v>
+      </c>
+      <c r="J2" t="s">
         <v>13</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H2" t="n">
-        <v>-6.06868760171146</v>
-      </c>
-      <c r="I2" t="n">
-        <v>38.4650393175249</v>
-      </c>
-      <c r="J2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46208</v>
+        <v>46212</v>
       </c>
       <c r="B3"/>
       <c r="C3" t="s">
@@ -493,83 +509,301 @@
       <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
+      <c r="E3"/>
       <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>19.1534851448814</v>
+      </c>
+      <c r="I3" t="n">
+        <v>39.9813771431375</v>
+      </c>
+      <c r="J3" t="s">
         <v>15</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-6.06868760171146</v>
-      </c>
-      <c r="I3" t="n">
-        <v>38.3750393175249</v>
-      </c>
-      <c r="J3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46208</v>
+        <v>46214</v>
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
+      <c r="E4"/>
       <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.0213661735589559</v>
+      </c>
+      <c r="I4" t="n">
+        <v>39.2333333333333</v>
+      </c>
+      <c r="J4" t="s">
         <v>13</v>
-      </c>
-      <c r="G4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.400685686389062</v>
-      </c>
-      <c r="I4" t="n">
-        <v>39.2392344497608</v>
-      </c>
-      <c r="J4" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46208</v>
+        <v>46214</v>
       </c>
       <c r="B5"/>
       <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5"/>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.0213661735589559</v>
+      </c>
+      <c r="I5" t="n">
+        <v>39.2333333333333</v>
+      </c>
+      <c r="J5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B6"/>
+      <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D6" t="s">
         <v>19</v>
       </c>
-      <c r="F5" t="s">
+      <c r="E6"/>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-6.6959330531643</v>
+      </c>
+      <c r="I6" t="n">
+        <v>35.3259592494485</v>
+      </c>
+      <c r="J6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B7"/>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7"/>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-6.6959330531643</v>
+      </c>
+      <c r="I7" t="n">
+        <v>35.3259592494485</v>
+      </c>
+      <c r="J7" t="s">
         <v>15</v>
       </c>
-      <c r="G5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.400685686389062</v>
-      </c>
-      <c r="I5" t="n">
-        <v>38.3392344497608</v>
-      </c>
-      <c r="J5" t="s">
-        <v>16</v>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B8"/>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8"/>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-7.37308900963752</v>
+      </c>
+      <c r="I8" t="n">
+        <v>44.9057402072379</v>
+      </c>
+      <c r="J8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B9"/>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9"/>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-7.37308900963752</v>
+      </c>
+      <c r="I9" t="n">
+        <v>44.9057402072379</v>
+      </c>
+      <c r="J9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B10"/>
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10"/>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8.11056950023961</v>
+      </c>
+      <c r="I10" t="n">
+        <v>39.9429973412096</v>
+      </c>
+      <c r="J10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B11"/>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11"/>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8.11056950023961</v>
+      </c>
+      <c r="I11" t="n">
+        <v>39.9429973412096</v>
+      </c>
+      <c r="J11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B12"/>
+      <c r="C12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12"/>
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3.56109503966957</v>
+      </c>
+      <c r="I12" t="n">
+        <v>40.4190254449825</v>
+      </c>
+      <c r="J12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B13"/>
+      <c r="C13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13"/>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3.56109503966957</v>
+      </c>
+      <c r="I13" t="n">
+        <v>40.4190254449825</v>
+      </c>
+      <c r="J13" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-07-11 12:05:25
</commit_message>
<xml_diff>
--- a/files/NRLW_upcoming_projections.xlsx
+++ b/files/NRLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -50,6 +50,9 @@
     <t xml:space="preserve">brisbane broncos</t>
   </si>
   <si>
+    <t xml:space="preserve">ocean protect stadium</t>
+  </si>
+  <si>
     <t xml:space="preserve">No Rain (Primary)</t>
   </si>
   <si>
@@ -68,28 +71,43 @@
     <t xml:space="preserve">gold coast titans</t>
   </si>
   <si>
+    <t xml:space="preserve">accor stadium</t>
+  </si>
+  <si>
     <t xml:space="preserve">north queensland cowboys</t>
   </si>
   <si>
     <t xml:space="preserve">wests tigers</t>
   </si>
   <si>
+    <t xml:space="preserve">queensland country bank stadium</t>
+  </si>
+  <si>
     <t xml:space="preserve">sydney roosters</t>
   </si>
   <si>
     <t xml:space="preserve">newcastle knights</t>
   </si>
   <si>
+    <t xml:space="preserve">allianz stadium</t>
+  </si>
+  <si>
     <t xml:space="preserve">canberra raiders</t>
   </si>
   <si>
     <t xml:space="preserve">warriors</t>
   </si>
   <si>
+    <t xml:space="preserve">gio stadium</t>
+  </si>
+  <si>
     <t xml:space="preserve">st george illawarra dragons</t>
   </si>
   <si>
     <t xml:space="preserve">parramatta eels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">win stadium</t>
   </si>
 </sst>
 </file>
@@ -430,7 +448,7 @@
     <col min="2" max="2" width="4.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="29.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="5.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="31.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="28.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
@@ -481,12 +499,14 @@
       <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="E2"/>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="H2" t="n">
         <v>19.1534851448814</v>
@@ -495,7 +515,7 @@
         <v>39.9813771431375</v>
       </c>
       <c r="J2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -509,21 +529,23 @@
       <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="E3"/>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="H3" t="n">
         <v>19.1534851448814</v>
       </c>
       <c r="I3" t="n">
-        <v>39.9813771431375</v>
+        <v>37.9413771431375</v>
       </c>
       <c r="J3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -532,14 +554,16 @@
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4"/>
+        <v>18</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -551,7 +575,7 @@
         <v>39.2333333333333</v>
       </c>
       <c r="J4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -560,14 +584,16 @@
       </c>
       <c r="B5"/>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5"/>
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -579,7 +605,7 @@
         <v>39.2333333333333</v>
       </c>
       <c r="J5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -588,14 +614,16 @@
       </c>
       <c r="B6"/>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6"/>
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
       <c r="F6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -607,7 +635,7 @@
         <v>35.3259592494485</v>
       </c>
       <c r="J6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -616,14 +644,16 @@
       </c>
       <c r="B7"/>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7"/>
+        <v>21</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -635,7 +665,7 @@
         <v>35.3259592494485</v>
       </c>
       <c r="J7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -644,14 +674,16 @@
       </c>
       <c r="B8"/>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8"/>
+        <v>24</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
+      </c>
       <c r="F8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -663,7 +695,7 @@
         <v>44.9057402072379</v>
       </c>
       <c r="J8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -672,14 +704,16 @@
       </c>
       <c r="B9"/>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9"/>
+        <v>24</v>
+      </c>
+      <c r="E9" t="s">
+        <v>25</v>
+      </c>
       <c r="F9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -691,7 +725,7 @@
         <v>44.9057402072379</v>
       </c>
       <c r="J9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -700,17 +734,19 @@
       </c>
       <c r="B10"/>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10"/>
+        <v>27</v>
+      </c>
+      <c r="E10" t="s">
+        <v>28</v>
+      </c>
       <c r="F10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="H10" t="n">
         <v>8.11056950023961</v>
@@ -719,7 +755,7 @@
         <v>39.9429973412096</v>
       </c>
       <c r="J10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -728,26 +764,28 @@
       </c>
       <c r="B11"/>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11"/>
+        <v>27</v>
+      </c>
+      <c r="E11" t="s">
+        <v>28</v>
+      </c>
       <c r="F11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="H11" t="n">
         <v>8.11056950023961</v>
       </c>
       <c r="I11" t="n">
-        <v>39.9429973412096</v>
+        <v>38.1729973412096</v>
       </c>
       <c r="J11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12">
@@ -756,14 +794,16 @@
       </c>
       <c r="B12"/>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12"/>
+        <v>30</v>
+      </c>
+      <c r="E12" t="s">
+        <v>31</v>
+      </c>
       <c r="F12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -775,7 +815,7 @@
         <v>40.4190254449825</v>
       </c>
       <c r="J12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -784,14 +824,16 @@
       </c>
       <c r="B13"/>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13"/>
+        <v>30</v>
+      </c>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
       <c r="F13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -803,7 +845,7 @@
         <v>40.4190254449825</v>
       </c>
       <c r="J13" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-07-16 16:26:28
</commit_message>
<xml_diff>
--- a/files/NRLW_upcoming_projections.xlsx
+++ b/files/NRLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,61 +44,70 @@
     <t xml:space="preserve">Weather Applied</t>
   </si>
   <si>
+    <t xml:space="preserve">canberra raiders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney roosters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gio stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain (Primary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No - primary model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted (Reference)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference only - heuristic -0.3 total pts/mm, cap +/-6</t>
+  </si>
+  <si>
     <t xml:space="preserve">canterbury bankstown bulldogs</t>
   </si>
   <si>
+    <t xml:space="preserve">cronulla-sutherland sharks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accor stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">warriors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north queensland cowboys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">go media stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane broncos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wests tigers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">totally workwear stadium</t>
+  </si>
+  <si>
     <t xml:space="preserve">gold coast titans</t>
   </si>
   <si>
-    <t xml:space="preserve">accor stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain (Primary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No - primary model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather Adjusted (Reference)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference only - heuristic -0.3 total pts/mm, cap +/-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north queensland cowboys</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wests tigers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">queensland country bank stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney roosters</t>
+    <t xml:space="preserve">parramatta eels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cbus super stadium</t>
   </si>
   <si>
     <t xml:space="preserve">newcastle knights</t>
   </si>
   <si>
-    <t xml:space="preserve">allianz stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">canberra raiders</t>
-  </si>
-  <si>
-    <t xml:space="preserve">warriors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gio stadium</t>
-  </si>
-  <si>
     <t xml:space="preserve">st george illawarra dragons</t>
   </si>
   <si>
-    <t xml:space="preserve">parramatta eels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">win stadium</t>
+    <t xml:space="preserve">mcdonald jones stadium</t>
   </si>
 </sst>
 </file>
@@ -438,8 +447,8 @@
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="4.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="29.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="31.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="27.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="24.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="28.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
@@ -481,7 +490,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B2"/>
       <c r="C2" t="s">
@@ -500,10 +509,10 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.643539734534159</v>
+        <v>20.4139838300442</v>
       </c>
       <c r="I2" t="n">
-        <v>39.2697674418605</v>
+        <v>46.4039632546516</v>
       </c>
       <c r="J2" t="s">
         <v>14</v>
@@ -511,7 +520,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B3"/>
       <c r="C3" t="s">
@@ -530,10 +539,10 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0.643539734534159</v>
+        <v>20.4139838300442</v>
       </c>
       <c r="I3" t="n">
-        <v>39.2697674418605</v>
+        <v>46.4039632546516</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -541,7 +550,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
@@ -557,13 +566,13 @@
         <v>13</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>-4.0919523812184</v>
+        <v>5.16988780313592</v>
       </c>
       <c r="I4" t="n">
-        <v>37.5696515092337</v>
+        <v>39.2697674418605</v>
       </c>
       <c r="J4" t="s">
         <v>14</v>
@@ -571,7 +580,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B5"/>
       <c r="C5" t="s">
@@ -587,13 +596,13 @@
         <v>15</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>-4.0919523812184</v>
+        <v>5.16988780313592</v>
       </c>
       <c r="I5" t="n">
-        <v>37.4796515092337</v>
+        <v>39.2697674418605</v>
       </c>
       <c r="J5" t="s">
         <v>16</v>
@@ -601,7 +610,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B6"/>
       <c r="C6" t="s">
@@ -620,10 +629,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>-6.93914962442005</v>
+        <v>-2.3474257695568</v>
       </c>
       <c r="I6" t="n">
-        <v>41.2678919464872</v>
+        <v>38.1359857396028</v>
       </c>
       <c r="J6" t="s">
         <v>14</v>
@@ -631,7 +640,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B7"/>
       <c r="C7" t="s">
@@ -650,10 +659,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>-6.93914962442005</v>
+        <v>-2.3474257695568</v>
       </c>
       <c r="I7" t="n">
-        <v>41.2678919464872</v>
+        <v>38.1359857396028</v>
       </c>
       <c r="J7" t="s">
         <v>16</v>
@@ -661,7 +670,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46215</v>
+        <v>46222</v>
       </c>
       <c r="B8"/>
       <c r="C8" t="s">
@@ -677,13 +686,13 @@
         <v>13</v>
       </c>
       <c r="G8" t="n">
-        <v>5.6</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>1.31285225907677</v>
+        <v>-31.1515608808005</v>
       </c>
       <c r="I8" t="n">
-        <v>43.5098321082488</v>
+        <v>43.8584480636318</v>
       </c>
       <c r="J8" t="s">
         <v>14</v>
@@ -691,7 +700,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46215</v>
+        <v>46222</v>
       </c>
       <c r="B9"/>
       <c r="C9" t="s">
@@ -707,13 +716,13 @@
         <v>15</v>
       </c>
       <c r="G9" t="n">
-        <v>5.6</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>1.31285225907677</v>
+        <v>-31.1515608808005</v>
       </c>
       <c r="I9" t="n">
-        <v>41.8298321082488</v>
+        <v>43.8584480636318</v>
       </c>
       <c r="J9" t="s">
         <v>16</v>
@@ -721,7 +730,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46215</v>
+        <v>46222</v>
       </c>
       <c r="B10"/>
       <c r="C10" t="s">
@@ -740,10 +749,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0.653061731611337</v>
+        <v>-3.96947877753608</v>
       </c>
       <c r="I10" t="n">
-        <v>38.3222898254997</v>
+        <v>36.6635543626358</v>
       </c>
       <c r="J10" t="s">
         <v>14</v>
@@ -751,7 +760,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46215</v>
+        <v>46222</v>
       </c>
       <c r="B11"/>
       <c r="C11" t="s">
@@ -770,12 +779,72 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>0.653061731611337</v>
+        <v>-3.96947877753608</v>
       </c>
       <c r="I11" t="n">
-        <v>38.3222898254997</v>
+        <v>36.6635543626358</v>
       </c>
       <c r="J11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B12"/>
+      <c r="C12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-12.645815833934</v>
+      </c>
+      <c r="I12" t="n">
+        <v>37.5095732369552</v>
+      </c>
+      <c r="J12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B13"/>
+      <c r="C13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-12.645815833934</v>
+      </c>
+      <c r="I13" t="n">
+        <v>37.5095732369552</v>
+      </c>
+      <c r="J13" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-07-25 12:40:47
</commit_message>
<xml_diff>
--- a/files/NRLW_upcoming_projections.xlsx
+++ b/files/NRLW_upcoming_projections.xlsx
@@ -44,70 +44,70 @@
     <t xml:space="preserve">Weather Applied</t>
   </si>
   <si>
+    <t xml:space="preserve">12:45</t>
+  </si>
+  <si>
     <t xml:space="preserve">canberra raiders</t>
   </si>
   <si>
+    <t xml:space="preserve">cronulla-sutherland sharks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain (Primary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No - primary model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted (Reference)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference only - heuristic -0.3 total pts/mm, cap +/-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">canterbury bankstown bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st george illawarra dragons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north queensland cowboys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast titans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane broncos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">newcastle knights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parramatta eels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">warriors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wests tigers</t>
+  </si>
+  <si>
     <t xml:space="preserve">sydney roosters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gio stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain (Primary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No - primary model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather Adjusted (Reference)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference only - heuristic -0.3 total pts/mm, cap +/-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">canterbury bankstown bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cronulla-sutherland sharks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">accor stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">warriors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north queensland cowboys</t>
-  </si>
-  <si>
-    <t xml:space="preserve">go media stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane broncos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wests tigers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">totally workwear stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast titans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parramatta eels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cbus super stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">newcastle knights</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st george illawarra dragons</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mcdonald jones stadium</t>
   </si>
 </sst>
 </file>
@@ -445,10 +445,10 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="4.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="29.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="27.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="24.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="5.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="28.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
@@ -490,18 +490,18 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B2"/>
+        <v>46228</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
         <v>12</v>
       </c>
+      <c r="E2"/>
       <c r="F2" t="s">
         <v>13</v>
       </c>
@@ -509,10 +509,10 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>20.4139838300442</v>
+        <v>-0.303507102607753</v>
       </c>
       <c r="I2" t="n">
-        <v>46.4039632546516</v>
+        <v>41.6289886221357</v>
       </c>
       <c r="J2" t="s">
         <v>14</v>
@@ -520,18 +520,18 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B3"/>
+        <v>46228</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
         <v>12</v>
       </c>
+      <c r="E3"/>
       <c r="F3" t="s">
         <v>15</v>
       </c>
@@ -539,10 +539,10 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>20.4139838300442</v>
+        <v>-0.303507102607753</v>
       </c>
       <c r="I3" t="n">
-        <v>46.4039632546516</v>
+        <v>41.6289886221357</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -550,18 +550,18 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B4"/>
+        <v>46228</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
         <v>19</v>
       </c>
+      <c r="E4"/>
       <c r="F4" t="s">
         <v>13</v>
       </c>
@@ -569,10 +569,10 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>5.16988780313592</v>
+        <v>0.983632499907437</v>
       </c>
       <c r="I4" t="n">
-        <v>39.2697674418605</v>
+        <v>41.7712962852712</v>
       </c>
       <c r="J4" t="s">
         <v>14</v>
@@ -580,18 +580,18 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B5"/>
+        <v>46228</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" t="s">
         <v>19</v>
       </c>
+      <c r="E5"/>
       <c r="F5" t="s">
         <v>15</v>
       </c>
@@ -599,10 +599,10 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>5.16988780313592</v>
+        <v>0.983632499907437</v>
       </c>
       <c r="I5" t="n">
-        <v>39.2697674418605</v>
+        <v>41.7712962852712</v>
       </c>
       <c r="J5" t="s">
         <v>16</v>
@@ -610,18 +610,18 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B6"/>
+        <v>46228</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" t="s">
         <v>22</v>
       </c>
+      <c r="E6"/>
       <c r="F6" t="s">
         <v>13</v>
       </c>
@@ -629,10 +629,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>-2.3474257695568</v>
+        <v>7.75404316407071</v>
       </c>
       <c r="I6" t="n">
-        <v>38.1359857396028</v>
+        <v>42.276371231609</v>
       </c>
       <c r="J6" t="s">
         <v>14</v>
@@ -640,18 +640,18 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B7"/>
+        <v>46228</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" t="s">
         <v>22</v>
       </c>
+      <c r="E7"/>
       <c r="F7" t="s">
         <v>15</v>
       </c>
@@ -659,10 +659,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>-2.3474257695568</v>
+        <v>7.75404316407071</v>
       </c>
       <c r="I7" t="n">
-        <v>38.1359857396028</v>
+        <v>42.276371231609</v>
       </c>
       <c r="J7" t="s">
         <v>16</v>
@@ -670,18 +670,18 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46222</v>
-      </c>
-      <c r="B8"/>
+        <v>46229</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" t="s">
         <v>25</v>
       </c>
+      <c r="E8"/>
       <c r="F8" t="s">
         <v>13</v>
       </c>
@@ -689,10 +689,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>-31.1515608808005</v>
+        <v>-7.41245114487048</v>
       </c>
       <c r="I8" t="n">
-        <v>43.8584480636318</v>
+        <v>42.7035756695531</v>
       </c>
       <c r="J8" t="s">
         <v>14</v>
@@ -700,18 +700,18 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46222</v>
-      </c>
-      <c r="B9"/>
+        <v>46229</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" t="s">
         <v>25</v>
       </c>
+      <c r="E9"/>
       <c r="F9" t="s">
         <v>15</v>
       </c>
@@ -719,10 +719,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>-31.1515608808005</v>
+        <v>-7.41245114487048</v>
       </c>
       <c r="I9" t="n">
-        <v>43.8584480636318</v>
+        <v>42.7035756695531</v>
       </c>
       <c r="J9" t="s">
         <v>16</v>
@@ -730,18 +730,18 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46222</v>
-      </c>
-      <c r="B10"/>
+        <v>46229</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" t="s">
         <v>28</v>
       </c>
+      <c r="E10"/>
       <c r="F10" t="s">
         <v>13</v>
       </c>
@@ -749,10 +749,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>-3.96947877753608</v>
+        <v>7.06506353550224</v>
       </c>
       <c r="I10" t="n">
-        <v>36.6635543626358</v>
+        <v>43.828153134857</v>
       </c>
       <c r="J10" t="s">
         <v>14</v>
@@ -760,18 +760,18 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46222</v>
-      </c>
-      <c r="B11"/>
+        <v>46229</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" t="s">
         <v>28</v>
       </c>
+      <c r="E11"/>
       <c r="F11" t="s">
         <v>15</v>
       </c>
@@ -779,10 +779,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>-3.96947877753608</v>
+        <v>7.06506353550224</v>
       </c>
       <c r="I11" t="n">
-        <v>36.6635543626358</v>
+        <v>43.828153134857</v>
       </c>
       <c r="J11" t="s">
         <v>16</v>
@@ -790,18 +790,18 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46222</v>
-      </c>
-      <c r="B12"/>
+        <v>46229</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" t="s">
         <v>31</v>
       </c>
+      <c r="E12"/>
       <c r="F12" t="s">
         <v>13</v>
       </c>
@@ -809,10 +809,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>-12.645815833934</v>
+        <v>13.6158206827388</v>
       </c>
       <c r="I12" t="n">
-        <v>37.5095732369552</v>
+        <v>42.1231998919844</v>
       </c>
       <c r="J12" t="s">
         <v>14</v>
@@ -820,18 +820,18 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46222</v>
-      </c>
-      <c r="B13"/>
+        <v>46229</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D13" t="s">
-        <v>30</v>
-      </c>
-      <c r="E13" t="s">
         <v>31</v>
       </c>
+      <c r="E13"/>
       <c r="F13" t="s">
         <v>15</v>
       </c>
@@ -839,10 +839,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>-12.645815833934</v>
+        <v>13.6158206827388</v>
       </c>
       <c r="I13" t="n">
-        <v>37.5095732369552</v>
+        <v>42.1231998919844</v>
       </c>
       <c r="J13" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
Update model outputs 2026-07-25 14:10:40
</commit_message>
<xml_diff>
--- a/files/NRLW_upcoming_projections.xlsx
+++ b/files/NRLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,70 +44,76 @@
     <t xml:space="preserve">Weather Applied</t>
   </si>
   <si>
-    <t xml:space="preserve">12:45</t>
+    <t xml:space="preserve">15:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">canterbury bankstown bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st george illawarra dragons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain (Primary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No - primary model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted (Reference)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference only - heuristic -0.3 total pts/mm, cap +/-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north queensland cowboys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast titans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane broncos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">newcastle knights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parramatta eels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">warriors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wests tigers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney roosters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:15</t>
   </si>
   <si>
     <t xml:space="preserve">canberra raiders</t>
   </si>
   <si>
+    <t xml:space="preserve">12:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">cronulla-sutherland sharks</t>
   </si>
   <si>
-    <t xml:space="preserve">No Rain (Primary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No - primary model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather Adjusted (Reference)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference only - heuristic -0.3 total pts/mm, cap +/-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">canterbury bankstown bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st george illawarra dragons</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north queensland cowboys</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast titans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane broncos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">newcastle knights</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parramatta eels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">warriors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wests tigers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney roosters</t>
+    <t xml:space="preserve">14:15</t>
   </si>
 </sst>
 </file>
@@ -509,10 +515,10 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.303507102607753</v>
+        <v>0.983632499907437</v>
       </c>
       <c r="I2" t="n">
-        <v>41.6289886221357</v>
+        <v>41.7712962852712</v>
       </c>
       <c r="J2" t="s">
         <v>14</v>
@@ -539,10 +545,10 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.303507102607753</v>
+        <v>0.983632499907437</v>
       </c>
       <c r="I3" t="n">
-        <v>41.6289886221357</v>
+        <v>41.7712962852712</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -569,10 +575,10 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>0.983632499907437</v>
+        <v>7.75404316407071</v>
       </c>
       <c r="I4" t="n">
-        <v>41.7712962852712</v>
+        <v>42.276371231609</v>
       </c>
       <c r="J4" t="s">
         <v>14</v>
@@ -599,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0.983632499907437</v>
+        <v>7.75404316407071</v>
       </c>
       <c r="I5" t="n">
-        <v>41.7712962852712</v>
+        <v>42.276371231609</v>
       </c>
       <c r="J5" t="s">
         <v>16</v>
@@ -610,7 +616,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -629,10 +635,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>7.75404316407071</v>
+        <v>-7.41245114487048</v>
       </c>
       <c r="I6" t="n">
-        <v>42.276371231609</v>
+        <v>42.7035756695531</v>
       </c>
       <c r="J6" t="s">
         <v>14</v>
@@ -640,7 +646,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
@@ -659,10 +665,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>7.75404316407071</v>
+        <v>-7.41245114487048</v>
       </c>
       <c r="I7" t="n">
-        <v>42.276371231609</v>
+        <v>42.7035756695531</v>
       </c>
       <c r="J7" t="s">
         <v>16</v>
@@ -689,10 +695,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>-7.41245114487048</v>
+        <v>7.06506353550224</v>
       </c>
       <c r="I8" t="n">
-        <v>42.7035756695531</v>
+        <v>43.828153134857</v>
       </c>
       <c r="J8" t="s">
         <v>14</v>
@@ -719,10 +725,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>-7.41245114487048</v>
+        <v>7.06506353550224</v>
       </c>
       <c r="I9" t="n">
-        <v>42.7035756695531</v>
+        <v>43.828153134857</v>
       </c>
       <c r="J9" t="s">
         <v>16</v>
@@ -749,10 +755,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>7.06506353550224</v>
+        <v>13.6158206827388</v>
       </c>
       <c r="I10" t="n">
-        <v>43.828153134857</v>
+        <v>42.1231998919844</v>
       </c>
       <c r="J10" t="s">
         <v>14</v>
@@ -779,10 +785,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>7.06506353550224</v>
+        <v>13.6158206827388</v>
       </c>
       <c r="I11" t="n">
-        <v>43.828153134857</v>
+        <v>42.1231998919844</v>
       </c>
       <c r="J11" t="s">
         <v>16</v>
@@ -790,7 +796,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46229</v>
+        <v>46235</v>
       </c>
       <c r="B12" t="s">
         <v>29</v>
@@ -799,7 +805,7 @@
         <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="E12"/>
       <c r="F12" t="s">
@@ -809,10 +815,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>13.6158206827388</v>
+        <v>-6.60121107254077</v>
       </c>
       <c r="I12" t="n">
-        <v>42.1231998919844</v>
+        <v>43.8126896797634</v>
       </c>
       <c r="J12" t="s">
         <v>14</v>
@@ -820,7 +826,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46229</v>
+        <v>46235</v>
       </c>
       <c r="B13" t="s">
         <v>29</v>
@@ -829,7 +835,7 @@
         <v>30</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="E13"/>
       <c r="F13" t="s">
@@ -839,12 +845,132 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>13.6158206827388</v>
+        <v>-6.60121107254077</v>
       </c>
       <c r="I13" t="n">
-        <v>42.1231998919844</v>
+        <v>43.8126896797634</v>
       </c>
       <c r="J13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14"/>
+      <c r="F14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-4.67780731917525</v>
+      </c>
+      <c r="I14" t="n">
+        <v>39.861449808901</v>
+      </c>
+      <c r="J14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15"/>
+      <c r="F15" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-4.67780731917525</v>
+      </c>
+      <c r="I15" t="n">
+        <v>39.861449808901</v>
+      </c>
+      <c r="J15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16"/>
+      <c r="F16" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>13.7837410781809</v>
+      </c>
+      <c r="I16" t="n">
+        <v>39.7411296607424</v>
+      </c>
+      <c r="J16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17"/>
+      <c r="F17" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>13.7837410781809</v>
+      </c>
+      <c r="I17" t="n">
+        <v>39.7411296607424</v>
+      </c>
+      <c r="J17" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-08-04 06:54:16
</commit_message>
<xml_diff>
--- a/files/NRLW_upcoming_projections.xlsx
+++ b/files/NRLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -38,6 +38,12 @@
     <t xml:space="preserve">Projected Total</t>
   </si>
   <si>
+    <t xml:space="preserve">Market Period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projection Type</t>
+  </si>
+  <si>
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
@@ -56,7 +62,16 @@
     <t xml:space="preserve">north queensland cowboys</t>
   </si>
   <si>
+    <t xml:space="preserve">FT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain (Primary)</t>
+  </si>
+  <si>
     <t xml:space="preserve">No - primary model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted (Reference)</t>
   </si>
   <si>
     <t xml:space="preserve">Reference only - heuristic -0.3 total pts/mm, cap +/-6</t>
@@ -449,9 +464,11 @@
     <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="15.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="5.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="16.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="54.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="13.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="28.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="5.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="16.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="54.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,19 +505,25 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
         <v>46242</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E2" t="n">
         <v>-0.967365923161965</v>
@@ -514,12 +537,18 @@
       <c r="H2" t="n">
         <v>41.1347508280856</v>
       </c>
-      <c r="I2"/>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="s">
-        <v>14</v>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2"/>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -527,13 +556,13 @@
         <v>46242</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
         <v>-0.967365923161965</v>
@@ -547,12 +576,18 @@
       <c r="H3" t="n">
         <v>41.1347508280856</v>
       </c>
-      <c r="I3"/>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="s">
-        <v>15</v>
+      <c r="I3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3"/>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -560,13 +595,13 @@
         <v>46242</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E4" t="n">
         <v>2.95591997136961</v>
@@ -580,12 +615,18 @@
       <c r="H4" t="n">
         <v>39.0546153809696</v>
       </c>
-      <c r="I4"/>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="s">
-        <v>14</v>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4"/>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -593,13 +634,13 @@
         <v>46242</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E5" t="n">
         <v>2.95591997136961</v>
@@ -613,12 +654,18 @@
       <c r="H5" t="n">
         <v>39.0546153809696</v>
       </c>
-      <c r="I5"/>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="s">
-        <v>15</v>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5"/>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -626,13 +673,13 @@
         <v>46242</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E6" t="n">
         <v>4.30523197794122</v>
@@ -646,12 +693,18 @@
       <c r="H6" t="n">
         <v>39.4395417954011</v>
       </c>
-      <c r="I6"/>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="s">
-        <v>14</v>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6"/>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -659,13 +712,13 @@
         <v>46242</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E7" t="n">
         <v>4.30523197794122</v>
@@ -679,12 +732,18 @@
       <c r="H7" t="n">
         <v>39.4395417954011</v>
       </c>
-      <c r="I7"/>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="s">
-        <v>15</v>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7"/>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -692,13 +751,13 @@
         <v>46243</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E8" t="n">
         <v>16.5034438582445</v>
@@ -712,12 +771,18 @@
       <c r="H8" t="n">
         <v>44.3103951350002</v>
       </c>
-      <c r="I8"/>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="s">
-        <v>14</v>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" t="s">
+        <v>17</v>
+      </c>
+      <c r="K8"/>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -725,13 +790,13 @@
         <v>46243</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E9" t="n">
         <v>16.5034438582445</v>
@@ -745,12 +810,18 @@
       <c r="H9" t="n">
         <v>44.3103951350002</v>
       </c>
-      <c r="I9"/>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="s">
-        <v>15</v>
+      <c r="I9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9"/>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -758,13 +829,13 @@
         <v>46243</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E10" t="n">
         <v>1.91884346032829</v>
@@ -778,12 +849,18 @@
       <c r="H10" t="n">
         <v>41.93872955763</v>
       </c>
-      <c r="I10"/>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="s">
-        <v>14</v>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10" t="s">
+        <v>17</v>
+      </c>
+      <c r="K10"/>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="11">
@@ -791,13 +868,13 @@
         <v>46243</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E11" t="n">
         <v>1.91884346032829</v>
@@ -811,12 +888,18 @@
       <c r="H11" t="n">
         <v>41.93872955763</v>
       </c>
-      <c r="I11"/>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="s">
-        <v>15</v>
+      <c r="I11" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K11"/>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="12">
@@ -824,13 +907,13 @@
         <v>46243</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E12" t="n">
         <v>-17.4666918131983</v>
@@ -844,12 +927,18 @@
       <c r="H12" t="n">
         <v>43.0792761429269</v>
       </c>
-      <c r="I12"/>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="s">
-        <v>14</v>
+      <c r="I12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J12" t="s">
+        <v>17</v>
+      </c>
+      <c r="K12"/>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -857,13 +946,13 @@
         <v>46243</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E13" t="n">
         <v>-17.4666918131983</v>
@@ -877,12 +966,18 @@
       <c r="H13" t="n">
         <v>43.0792761429269</v>
       </c>
-      <c r="I13"/>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="s">
-        <v>15</v>
+      <c r="I13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K13"/>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>